<commit_message>
Organize SickKids analysis files
</commit_message>
<xml_diff>
--- a/Anvio/07_PANGENOMICS/pathway_enrichment_pangenome.xlsx
+++ b/Anvio/07_PANGENOMICS/pathway_enrichment_pangenome.xlsx
@@ -8,16 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielcm/Desktop/SickKids/Anvio/07_PANGENOMICS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFE052B-B51F-B84E-9C5A-DD62C3EA20F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86B34BA-337B-9C4E-918A-6059BC67900B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="19200" windowHeight="21100" xr2:uid="{1F968237-E306-C946-BF9F-63DAE5DA727A}"/>
+    <workbookView xWindow="-35840" yWindow="0" windowWidth="35840" windowHeight="22400" activeTab="2" xr2:uid="{1F968237-E306-C946-BF9F-63DAE5DA727A}"/>
   </bookViews>
   <sheets>
     <sheet name="NS1 w9w10 enrichment" sheetId="1" r:id="rId1"/>
     <sheet name="S2 w9w10 enrichment" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NS1 w9w10 enrichment'!$A$1:$A$143</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="279">
   <si>
     <t>Shared taxa in NS, S</t>
   </si>
@@ -347,9 +350,6 @@
   </si>
   <si>
     <t>PWY0-41 (E. coli)</t>
-  </si>
-  <si>
-    <t>The strain of NS1 is the only one capable to complete this pathway. Pangenome differences suggest enrichment could be attributed to this.</t>
   </si>
   <si>
     <t>E. bolteae, E. citroniae</t>
@@ -773,9 +773,6 @@
     </r>
   </si>
   <si>
-    <t>There is evidence to suggest the pangenome differences could be driving the enrichment. However, if eggnog is right, then there is a product imbalance where S has all products but NS does not.</t>
-  </si>
-  <si>
     <t>1.1.1.49</t>
   </si>
   <si>
@@ -837,9 +834,6 @@
   </si>
   <si>
     <t>The pathways between all isolates are identical by anvi'o annotation but not by eggnog. If we use Anvi'o as reference, then there is no production of S-lactate, and only R-lactate for all 5 strains, and both have two routes of entry. But if we use eggnog's annotation, then the two seroconverted strains then S produced both products but NS does not.</t>
-  </si>
-  <si>
-    <t>Potential pangenome differences when using eggNOG mapper as a tool, but not when using Anvi'os profile.</t>
   </si>
   <si>
     <t>4.2.1.151</t>
@@ -1191,6 +1185,9 @@
   </si>
   <si>
     <t>There is no evidence to suggest pangenome differences are driving enrichment.</t>
+  </si>
+  <si>
+    <t>There is evidence to suggest that the pangenome has the potential to be driving some differences in enrichment</t>
   </si>
 </sst>
 </file>
@@ -1502,7 +1499,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1852,13 +1870,13 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="F1" s="36" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G1" s="36"/>
       <c r="H1" s="36"/>
       <c r="I1" s="36"/>
       <c r="J1" s="36" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K1" s="36"/>
       <c r="L1" s="36"/>
@@ -1952,10 +1970,10 @@
         <v>1</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -2209,10 +2227,10 @@
         <v>1</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -2676,10 +2694,10 @@
         <v>1</v>
       </c>
       <c r="N23" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O23" s="18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
@@ -2866,7 +2884,7 @@
         <v>39</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
@@ -3015,10 +3033,10 @@
         <v>1</v>
       </c>
       <c r="N32" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O32" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
@@ -3167,10 +3185,10 @@
         <v>1</v>
       </c>
       <c r="N36" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="O36" s="9" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
@@ -3564,10 +3582,10 @@
         <v>1</v>
       </c>
       <c r="N47" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O47" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.2">
@@ -3821,10 +3839,10 @@
         <v>0</v>
       </c>
       <c r="N54" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O54" s="9" t="s">
-        <v>102</v>
+        <v>276</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.2">
@@ -4148,10 +4166,10 @@
         <v>0</v>
       </c>
       <c r="N63" s="18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O63" s="18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.2">
@@ -4405,10 +4423,10 @@
         <v>0</v>
       </c>
       <c r="N70" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O70" s="9" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.2">
@@ -4592,10 +4610,10 @@
         <v>0</v>
       </c>
       <c r="N75" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O75" s="18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.2">
@@ -4954,10 +4972,10 @@
         <v>1</v>
       </c>
       <c r="N85" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O85" s="9" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.2">
@@ -5353,7 +5371,7 @@
         <v>14</v>
       </c>
       <c r="C97" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D97" s="17" t="s">
         <v>79</v>
@@ -5386,10 +5404,10 @@
         <v>1</v>
       </c>
       <c r="N97" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O97" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.2">
@@ -5849,13 +5867,13 @@
     </row>
     <row r="111" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B111" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D111" s="8" t="s">
         <v>93</v>
@@ -5888,10 +5906,10 @@
         <v>1</v>
       </c>
       <c r="N111" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.2">
@@ -6071,13 +6089,13 @@
     </row>
     <row r="117" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B117" s="21" t="s">
         <v>14</v>
       </c>
       <c r="C117" s="22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D117" s="17" t="s">
         <v>93</v>
@@ -6110,10 +6128,10 @@
         <v>1</v>
       </c>
       <c r="N117" s="23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O117" s="23" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.2">
@@ -6293,16 +6311,16 @@
     </row>
     <row r="123" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A123" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B123" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C123" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D123" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E123" s="6" t="s">
         <v>38</v>
@@ -6332,10 +6350,10 @@
         <v>1</v>
       </c>
       <c r="N123" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="O123" s="9" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="124" spans="1:15" x14ac:dyDescent="0.2">
@@ -6343,7 +6361,7 @@
       <c r="B124" s="6"/>
       <c r="C124" s="6"/>
       <c r="D124" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E124" s="6"/>
       <c r="F124" s="8">
@@ -6378,7 +6396,7 @@
       <c r="B125" s="6"/>
       <c r="C125" s="6"/>
       <c r="D125" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E125" s="6"/>
       <c r="F125" s="8">
@@ -6413,7 +6431,7 @@
       <c r="B126" s="6"/>
       <c r="C126" s="6"/>
       <c r="D126" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E126" s="6"/>
       <c r="F126" s="8">
@@ -6448,7 +6466,7 @@
       <c r="B127" s="6"/>
       <c r="C127" s="6"/>
       <c r="D127" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E127" s="6"/>
       <c r="F127" s="8">
@@ -6483,7 +6501,7 @@
       <c r="B128" s="6"/>
       <c r="C128" s="6"/>
       <c r="D128" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E128" s="6"/>
       <c r="F128" s="13">
@@ -6518,7 +6536,7 @@
       <c r="B129" s="6"/>
       <c r="C129" s="6"/>
       <c r="D129" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E129" s="6"/>
       <c r="F129" s="13">
@@ -6550,16 +6568,16 @@
     </row>
     <row r="130" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A130" s="18" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B130" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C130" s="18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D130" s="17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E130" s="18" t="s">
         <v>38</v>
@@ -6589,10 +6607,10 @@
         <v>75</v>
       </c>
       <c r="N130" s="18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O130" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="131" spans="1:15" x14ac:dyDescent="0.2">
@@ -6600,7 +6618,7 @@
       <c r="B131" s="18"/>
       <c r="C131" s="18"/>
       <c r="D131" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E131" s="18"/>
       <c r="F131" s="17">
@@ -6635,7 +6653,7 @@
       <c r="B132" s="18"/>
       <c r="C132" s="18"/>
       <c r="D132" s="17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E132" s="18"/>
       <c r="F132" s="17">
@@ -6670,7 +6688,7 @@
       <c r="B133" s="18"/>
       <c r="C133" s="18"/>
       <c r="D133" s="17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E133" s="18"/>
       <c r="F133" s="17">
@@ -6705,7 +6723,7 @@
       <c r="B134" s="18"/>
       <c r="C134" s="18"/>
       <c r="D134" s="17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E134" s="18"/>
       <c r="F134" s="19">
@@ -6740,7 +6758,7 @@
       <c r="B135" s="18"/>
       <c r="C135" s="18"/>
       <c r="D135" s="17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E135" s="18"/>
       <c r="F135" s="19">
@@ -6775,7 +6793,7 @@
       <c r="B136" s="18"/>
       <c r="C136" s="18"/>
       <c r="D136" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E136" s="18"/>
       <c r="F136" s="19">
@@ -6846,10 +6864,10 @@
         <v>1</v>
       </c>
       <c r="N137" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O137" s="9" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="138" spans="1:15" x14ac:dyDescent="0.2">
@@ -7063,6 +7081,7 @@
       <c r="O143" s="9"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A143" xr:uid="{CB553C35-DF1C-6B44-B066-1DB3F87C301B}"/>
   <mergeCells count="110">
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="J1:M1"/>
@@ -7204,13 +7223,13 @@
       <c r="D1" s="35"/>
       <c r="E1" s="35"/>
       <c r="F1" s="36" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G1" s="36"/>
       <c r="H1" s="36"/>
       <c r="I1" s="36"/>
       <c r="J1" s="36" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K1" s="36"/>
       <c r="L1" s="36"/>
@@ -7229,7 +7248,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="38" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E2" s="37" t="s">
         <v>2</v>
@@ -7267,16 +7286,16 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>134</v>
-      </c>
       <c r="D3" s="17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>23</v>
@@ -7306,10 +7325,10 @@
         <v>1</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>148</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -7317,7 +7336,7 @@
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
       <c r="D4" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E4" s="14"/>
       <c r="F4" s="19">
@@ -7352,7 +7371,7 @@
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
       <c r="D5" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="19">
@@ -7387,7 +7406,7 @@
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
       <c r="D6" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="19">
@@ -7422,7 +7441,7 @@
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
       <c r="D7" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="19">
@@ -7457,7 +7476,7 @@
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
       <c r="D8" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="19">
@@ -7492,7 +7511,7 @@
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
       <c r="D9" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="19">
@@ -7524,16 +7543,16 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>23</v>
@@ -7563,10 +7582,10 @@
         <v>1</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>170</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -7574,7 +7593,7 @@
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="10">
@@ -7609,7 +7628,7 @@
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="10">
@@ -7644,7 +7663,7 @@
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="10">
@@ -7679,7 +7698,7 @@
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="10">
@@ -7714,7 +7733,7 @@
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
       <c r="D15" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="10">
@@ -7749,7 +7768,7 @@
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="8" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E16" s="6"/>
       <c r="F16" s="10">
@@ -7784,7 +7803,7 @@
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E17" s="6"/>
       <c r="F17" s="10">
@@ -7819,7 +7838,7 @@
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="10">
@@ -7854,7 +7873,7 @@
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="10">
@@ -7889,7 +7908,7 @@
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="10">
@@ -7924,7 +7943,7 @@
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="10">
@@ -7959,7 +7978,7 @@
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="10">
@@ -7994,7 +8013,7 @@
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="10">
@@ -8029,7 +8048,7 @@
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="10">
@@ -8064,7 +8083,7 @@
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="10">
@@ -8099,7 +8118,7 @@
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="10">
@@ -8131,16 +8150,16 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E27" s="18" t="s">
         <v>38</v>
@@ -8170,10 +8189,10 @@
         <v>1</v>
       </c>
       <c r="N27" s="18" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="O27" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
@@ -8181,7 +8200,7 @@
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
       <c r="D28" s="17" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E28" s="18"/>
       <c r="F28" s="19">
@@ -8216,7 +8235,7 @@
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
       <c r="D29" s="17" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E29" s="18"/>
       <c r="F29" s="19">
@@ -8251,7 +8270,7 @@
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
       <c r="D30" s="17" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E30" s="18"/>
       <c r="F30" s="19">
@@ -8286,7 +8305,7 @@
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
       <c r="D31" s="17" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E31" s="18"/>
       <c r="F31" s="19">
@@ -8318,16 +8337,16 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>139</v>
-      </c>
       <c r="D32" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>38</v>
@@ -8357,10 +8376,10 @@
         <v>1</v>
       </c>
       <c r="N32" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="O32" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
@@ -8368,7 +8387,7 @@
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="10">
@@ -8403,7 +8422,7 @@
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
       <c r="D34" s="8" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E34" s="9"/>
       <c r="F34" s="10">
@@ -8438,7 +8457,7 @@
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
       <c r="D35" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="10">
@@ -8473,7 +8492,7 @@
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
       <c r="D36" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="10">
@@ -8508,7 +8527,7 @@
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="8" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="10">
@@ -8540,19 +8559,19 @@
     </row>
     <row r="38" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="18" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C38" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="D38" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="D38" s="17" t="s">
-        <v>184</v>
-      </c>
       <c r="E38" s="18" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F38" s="19">
         <v>0</v>
@@ -8579,10 +8598,10 @@
         <v>0</v>
       </c>
       <c r="N38" s="18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="O38" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
@@ -8590,7 +8609,7 @@
       <c r="B39" s="18"/>
       <c r="C39" s="18"/>
       <c r="D39" s="17" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E39" s="18"/>
       <c r="F39" s="19">
@@ -8625,7 +8644,7 @@
       <c r="B40" s="18"/>
       <c r="C40" s="18"/>
       <c r="D40" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E40" s="18"/>
       <c r="F40" s="19">
@@ -8660,7 +8679,7 @@
       <c r="B41" s="18"/>
       <c r="C41" s="18"/>
       <c r="D41" s="17" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E41" s="18"/>
       <c r="F41" s="19">
@@ -8695,7 +8714,7 @@
       <c r="B42" s="18"/>
       <c r="C42" s="18"/>
       <c r="D42" s="17" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E42" s="18"/>
       <c r="F42" s="19">
@@ -8730,7 +8749,7 @@
       <c r="B43" s="18"/>
       <c r="C43" s="18"/>
       <c r="D43" s="17" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E43" s="18"/>
       <c r="F43" s="19">
@@ -8765,7 +8784,7 @@
       <c r="B44" s="18"/>
       <c r="C44" s="18"/>
       <c r="D44" s="17" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E44" s="18"/>
       <c r="F44" s="19">
@@ -8800,7 +8819,7 @@
       <c r="B45" s="18"/>
       <c r="C45" s="18"/>
       <c r="D45" s="17" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E45" s="18"/>
       <c r="F45" s="19">
@@ -8835,7 +8854,7 @@
       <c r="B46" s="18"/>
       <c r="C46" s="18"/>
       <c r="D46" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E46" s="18"/>
       <c r="F46" s="19">
@@ -8867,16 +8886,16 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>38</v>
@@ -8906,10 +8925,10 @@
         <v>1</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.2">
@@ -8917,7 +8936,7 @@
       <c r="B48" s="9"/>
       <c r="C48" s="9"/>
       <c r="D48" s="8" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E48" s="9"/>
       <c r="F48" s="10">
@@ -8952,7 +8971,7 @@
       <c r="B49" s="9"/>
       <c r="C49" s="9"/>
       <c r="D49" s="8" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E49" s="9"/>
       <c r="F49" s="10">
@@ -8987,7 +9006,7 @@
       <c r="B50" s="9"/>
       <c r="C50" s="9"/>
       <c r="D50" s="8" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E50" s="9"/>
       <c r="F50" s="10">
@@ -9022,7 +9041,7 @@
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
       <c r="D51" s="8" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E51" s="9"/>
       <c r="F51" s="10">
@@ -9054,13 +9073,13 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C52" s="18" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D52" s="17" t="s">
         <v>67</v>
@@ -9093,10 +9112,10 @@
         <v>1</v>
       </c>
       <c r="N52" s="18" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="O52" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.2">
@@ -9209,7 +9228,7 @@
       <c r="B56" s="18"/>
       <c r="C56" s="18"/>
       <c r="D56" s="17" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E56" s="18"/>
       <c r="F56" s="19">
@@ -9244,7 +9263,7 @@
       <c r="B57" s="18"/>
       <c r="C57" s="18"/>
       <c r="D57" s="17" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E57" s="18"/>
       <c r="F57" s="19">
@@ -9279,7 +9298,7 @@
       <c r="B58" s="18"/>
       <c r="C58" s="18"/>
       <c r="D58" s="17" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E58" s="18"/>
       <c r="F58" s="19">
@@ -9384,7 +9403,7 @@
       <c r="B61" s="18"/>
       <c r="C61" s="18"/>
       <c r="D61" s="17" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E61" s="18"/>
       <c r="F61" s="19">
@@ -9419,7 +9438,7 @@
       <c r="B62" s="18"/>
       <c r="C62" s="18"/>
       <c r="D62" s="17" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E62" s="18"/>
       <c r="F62" s="19">
@@ -9454,7 +9473,7 @@
       <c r="B63" s="18"/>
       <c r="C63" s="18"/>
       <c r="D63" s="17" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E63" s="18"/>
       <c r="F63" s="19">
@@ -9489,7 +9508,7 @@
       <c r="B64" s="18"/>
       <c r="C64" s="18"/>
       <c r="D64" s="17" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E64" s="18"/>
       <c r="F64" s="19">
@@ -9524,7 +9543,7 @@
       <c r="B65" s="18"/>
       <c r="C65" s="18"/>
       <c r="D65" s="17" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E65" s="18"/>
       <c r="F65" s="19">
@@ -9559,7 +9578,7 @@
       <c r="B66" s="18"/>
       <c r="C66" s="18"/>
       <c r="D66" s="17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E66" s="18"/>
       <c r="F66" s="19">
@@ -9594,7 +9613,7 @@
       <c r="B67" s="18"/>
       <c r="C67" s="18"/>
       <c r="D67" s="17" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E67" s="18"/>
       <c r="F67" s="19">
@@ -9629,7 +9648,7 @@
       <c r="B68" s="18"/>
       <c r="C68" s="18"/>
       <c r="D68" s="17" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E68" s="18"/>
       <c r="F68" s="19">
@@ -9661,13 +9680,13 @@
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>67</v>
@@ -9700,10 +9719,10 @@
         <v>1</v>
       </c>
       <c r="N69" s="46" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="O69" s="46" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.2">
@@ -9816,7 +9835,7 @@
       <c r="B73" s="9"/>
       <c r="C73" s="9"/>
       <c r="D73" s="8" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E73" s="9"/>
       <c r="F73" s="12">
@@ -9851,7 +9870,7 @@
       <c r="B74" s="9"/>
       <c r="C74" s="9"/>
       <c r="D74" s="8" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E74" s="9"/>
       <c r="F74" s="12">
@@ -9886,7 +9905,7 @@
       <c r="B75" s="9"/>
       <c r="C75" s="9"/>
       <c r="D75" s="8" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E75" s="9"/>
       <c r="F75" s="12">
@@ -9991,7 +10010,7 @@
       <c r="B78" s="9"/>
       <c r="C78" s="9"/>
       <c r="D78" s="8" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E78" s="9"/>
       <c r="F78" s="12">
@@ -10026,7 +10045,7 @@
       <c r="B79" s="9"/>
       <c r="C79" s="9"/>
       <c r="D79" s="8" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E79" s="9"/>
       <c r="F79" s="12">
@@ -10061,7 +10080,7 @@
       <c r="B80" s="9"/>
       <c r="C80" s="9"/>
       <c r="D80" s="8" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E80" s="9"/>
       <c r="F80" s="12">
@@ -10096,7 +10115,7 @@
       <c r="B81" s="9"/>
       <c r="C81" s="9"/>
       <c r="D81" s="8" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E81" s="9"/>
       <c r="F81" s="12">
@@ -10131,7 +10150,7 @@
       <c r="B82" s="9"/>
       <c r="C82" s="9"/>
       <c r="D82" s="8" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E82" s="9"/>
       <c r="F82" s="12">
@@ -10166,7 +10185,7 @@
       <c r="B83" s="9"/>
       <c r="C83" s="9"/>
       <c r="D83" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E83" s="9"/>
       <c r="F83" s="12">
@@ -10201,7 +10220,7 @@
       <c r="B84" s="9"/>
       <c r="C84" s="9"/>
       <c r="D84" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E84" s="9"/>
       <c r="F84" s="12">
@@ -10236,7 +10255,7 @@
       <c r="B85" s="9"/>
       <c r="C85" s="9"/>
       <c r="D85" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E85" s="9"/>
       <c r="F85" s="12">
@@ -10268,16 +10287,16 @@
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A86" s="18" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B86" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C86" s="18" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D86" s="17" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E86" s="18" t="s">
         <v>38</v>
@@ -10307,10 +10326,10 @@
         <v>0</v>
       </c>
       <c r="N86" s="18" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="O86" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.2">
@@ -10318,7 +10337,7 @@
       <c r="B87" s="18"/>
       <c r="C87" s="18"/>
       <c r="D87" s="17" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E87" s="18"/>
       <c r="F87" s="19">
@@ -10353,7 +10372,7 @@
       <c r="B88" s="18"/>
       <c r="C88" s="18"/>
       <c r="D88" s="17" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E88" s="18"/>
       <c r="F88" s="19">
@@ -10388,7 +10407,7 @@
       <c r="B89" s="18"/>
       <c r="C89" s="18"/>
       <c r="D89" s="17" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E89" s="18"/>
       <c r="F89" s="19">
@@ -10423,7 +10442,7 @@
       <c r="B90" s="18"/>
       <c r="C90" s="18"/>
       <c r="D90" s="17" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E90" s="18"/>
       <c r="F90" s="19">
@@ -10455,16 +10474,16 @@
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A91" s="9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C91" s="9" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>38</v>
@@ -10494,10 +10513,10 @@
         <v>0</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.2">
@@ -10505,7 +10524,7 @@
       <c r="B92" s="9"/>
       <c r="C92" s="9"/>
       <c r="D92" s="8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E92" s="9"/>
       <c r="F92" s="12">
@@ -10540,7 +10559,7 @@
       <c r="B93" s="9"/>
       <c r="C93" s="9"/>
       <c r="D93" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E93" s="9"/>
       <c r="F93" s="12">
@@ -10575,7 +10594,7 @@
       <c r="B94" s="9"/>
       <c r="C94" s="9"/>
       <c r="D94" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E94" s="9"/>
       <c r="F94" s="12">
@@ -10610,7 +10629,7 @@
       <c r="B95" s="9"/>
       <c r="C95" s="9"/>
       <c r="D95" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E95" s="9"/>
       <c r="F95" s="12">
@@ -10642,16 +10661,16 @@
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A96" s="18" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B96" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C96" s="18" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D96" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E96" s="18" t="s">
         <v>38</v>
@@ -10681,10 +10700,10 @@
         <v>1</v>
       </c>
       <c r="N96" s="18" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="O96" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.2">
@@ -10692,7 +10711,7 @@
       <c r="B97" s="18"/>
       <c r="C97" s="18"/>
       <c r="D97" s="17" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E97" s="18"/>
       <c r="F97" s="19">
@@ -10727,7 +10746,7 @@
       <c r="B98" s="18"/>
       <c r="C98" s="18"/>
       <c r="D98" s="17" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E98" s="18"/>
       <c r="F98" s="19">
@@ -10762,7 +10781,7 @@
       <c r="B99" s="18"/>
       <c r="C99" s="18"/>
       <c r="D99" s="17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E99" s="18"/>
       <c r="F99" s="19">
@@ -10797,32 +10816,32 @@
       <c r="B100" s="18"/>
       <c r="C100" s="18"/>
       <c r="D100" s="17" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E100" s="18"/>
       <c r="F100" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G100" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H100" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I100" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J100" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K100" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L100" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M100" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N100" s="18"/>
       <c r="O100" s="18"/>
@@ -10832,7 +10851,7 @@
       <c r="B101" s="18"/>
       <c r="C101" s="18"/>
       <c r="D101" s="17" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E101" s="18"/>
       <c r="F101" s="19">
@@ -10867,7 +10886,7 @@
       <c r="B102" s="18"/>
       <c r="C102" s="18"/>
       <c r="D102" s="17" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E102" s="18"/>
       <c r="F102" s="19">
@@ -10902,7 +10921,7 @@
       <c r="B103" s="18"/>
       <c r="C103" s="18"/>
       <c r="D103" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E103" s="18"/>
       <c r="F103" s="19">
@@ -10934,16 +10953,16 @@
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A104" s="9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B104" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C104" s="9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D104" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E104" s="9" t="s">
         <v>38</v>
@@ -10973,10 +10992,10 @@
         <v>1</v>
       </c>
       <c r="N104" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="O104" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.2">
@@ -10984,7 +11003,7 @@
       <c r="B105" s="9"/>
       <c r="C105" s="9"/>
       <c r="D105" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E105" s="9"/>
       <c r="F105" s="12">
@@ -11019,7 +11038,7 @@
       <c r="B106" s="9"/>
       <c r="C106" s="9"/>
       <c r="D106" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E106" s="9"/>
       <c r="F106" s="12">
@@ -11054,7 +11073,7 @@
       <c r="B107" s="9"/>
       <c r="C107" s="9"/>
       <c r="D107" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E107" s="9"/>
       <c r="F107" s="12">
@@ -11089,32 +11108,32 @@
       <c r="B108" s="9"/>
       <c r="C108" s="9"/>
       <c r="D108" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E108" s="9"/>
       <c r="F108" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G108" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H108" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I108" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J108" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K108" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L108" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M108" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N108" s="9"/>
       <c r="O108" s="9"/>
@@ -11124,7 +11143,7 @@
       <c r="B109" s="9"/>
       <c r="C109" s="9"/>
       <c r="D109" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E109" s="9"/>
       <c r="F109" s="12">
@@ -11159,7 +11178,7 @@
       <c r="B110" s="9"/>
       <c r="C110" s="9"/>
       <c r="D110" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E110" s="9"/>
       <c r="F110" s="12">
@@ -11194,7 +11213,7 @@
       <c r="B111" s="9"/>
       <c r="C111" s="9"/>
       <c r="D111" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E111" s="9"/>
       <c r="F111" s="12">
@@ -11226,16 +11245,16 @@
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A112" s="18" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B112" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C112" s="18" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D112" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E112" s="18" t="s">
         <v>38</v>
@@ -11265,10 +11284,10 @@
         <v>1</v>
       </c>
       <c r="N112" s="18" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="O112" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.2">
@@ -11276,7 +11295,7 @@
       <c r="B113" s="18"/>
       <c r="C113" s="18"/>
       <c r="D113" s="17" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E113" s="18"/>
       <c r="F113" s="19">
@@ -11311,7 +11330,7 @@
       <c r="B114" s="18"/>
       <c r="C114" s="18"/>
       <c r="D114" s="17" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E114" s="18"/>
       <c r="F114" s="19">
@@ -11346,7 +11365,7 @@
       <c r="B115" s="18"/>
       <c r="C115" s="18"/>
       <c r="D115" s="17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E115" s="18"/>
       <c r="F115" s="19">
@@ -11381,32 +11400,32 @@
       <c r="B116" s="18"/>
       <c r="C116" s="18"/>
       <c r="D116" s="17" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E116" s="18"/>
       <c r="F116" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G116" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H116" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I116" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J116" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K116" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L116" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M116" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N116" s="18"/>
       <c r="O116" s="18"/>
@@ -11416,7 +11435,7 @@
       <c r="B117" s="18"/>
       <c r="C117" s="18"/>
       <c r="D117" s="17" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E117" s="18"/>
       <c r="F117" s="19">
@@ -11451,7 +11470,7 @@
       <c r="B118" s="18"/>
       <c r="C118" s="18"/>
       <c r="D118" s="17" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E118" s="18"/>
       <c r="F118" s="19">
@@ -11486,7 +11505,7 @@
       <c r="B119" s="18"/>
       <c r="C119" s="18"/>
       <c r="D119" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E119" s="18"/>
       <c r="F119" s="19">
@@ -11518,16 +11537,16 @@
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A120" s="9" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B120" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C120" s="9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D120" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E120" s="9" t="s">
         <v>38</v>
@@ -11557,10 +11576,10 @@
         <v>1</v>
       </c>
       <c r="N120" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="O120" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="121" spans="1:15" x14ac:dyDescent="0.2">
@@ -11568,7 +11587,7 @@
       <c r="B121" s="9"/>
       <c r="C121" s="9"/>
       <c r="D121" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E121" s="9"/>
       <c r="F121" s="12">
@@ -11603,7 +11622,7 @@
       <c r="B122" s="9"/>
       <c r="C122" s="9"/>
       <c r="D122" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E122" s="9"/>
       <c r="F122" s="12">
@@ -11638,7 +11657,7 @@
       <c r="B123" s="9"/>
       <c r="C123" s="9"/>
       <c r="D123" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E123" s="9"/>
       <c r="F123" s="12">
@@ -11673,32 +11692,32 @@
       <c r="B124" s="9"/>
       <c r="C124" s="9"/>
       <c r="D124" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E124" s="9"/>
       <c r="F124" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G124" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I124" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J124" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K124" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L124" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M124" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N124" s="9"/>
       <c r="O124" s="9"/>
@@ -11708,7 +11727,7 @@
       <c r="B125" s="9"/>
       <c r="C125" s="9"/>
       <c r="D125" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E125" s="9"/>
       <c r="F125" s="12">
@@ -11743,7 +11762,7 @@
       <c r="B126" s="9"/>
       <c r="C126" s="9"/>
       <c r="D126" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E126" s="9"/>
       <c r="F126" s="12">
@@ -11778,7 +11797,7 @@
       <c r="B127" s="9"/>
       <c r="C127" s="9"/>
       <c r="D127" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E127" s="9"/>
       <c r="F127" s="12">
@@ -11810,16 +11829,16 @@
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A128" s="18" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B128" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C128" s="18" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D128" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E128" s="18" t="s">
         <v>38</v>
@@ -11849,10 +11868,10 @@
         <v>1</v>
       </c>
       <c r="N128" s="18" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="O128" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="129" spans="1:15" x14ac:dyDescent="0.2">
@@ -11860,7 +11879,7 @@
       <c r="B129" s="18"/>
       <c r="C129" s="18"/>
       <c r="D129" s="17" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E129" s="18"/>
       <c r="F129" s="19">
@@ -11895,7 +11914,7 @@
       <c r="B130" s="18"/>
       <c r="C130" s="18"/>
       <c r="D130" s="17" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E130" s="18"/>
       <c r="F130" s="19">
@@ -11930,7 +11949,7 @@
       <c r="B131" s="18"/>
       <c r="C131" s="18"/>
       <c r="D131" s="17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E131" s="18"/>
       <c r="F131" s="19">
@@ -11965,32 +11984,32 @@
       <c r="B132" s="18"/>
       <c r="C132" s="18"/>
       <c r="D132" s="17" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E132" s="18"/>
       <c r="F132" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G132" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H132" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I132" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J132" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K132" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L132" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M132" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N132" s="18"/>
       <c r="O132" s="18"/>
@@ -12000,7 +12019,7 @@
       <c r="B133" s="18"/>
       <c r="C133" s="18"/>
       <c r="D133" s="17" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E133" s="18"/>
       <c r="F133" s="19">
@@ -12035,7 +12054,7 @@
       <c r="B134" s="18"/>
       <c r="C134" s="18"/>
       <c r="D134" s="17" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E134" s="18"/>
       <c r="F134" s="19">
@@ -12070,7 +12089,7 @@
       <c r="B135" s="18"/>
       <c r="C135" s="18"/>
       <c r="D135" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E135" s="18"/>
       <c r="F135" s="19">
@@ -12102,16 +12121,16 @@
     </row>
     <row r="136" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A136" s="9" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B136" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C136" s="9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D136" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E136" s="9" t="s">
         <v>38</v>
@@ -12141,10 +12160,10 @@
         <v>1</v>
       </c>
       <c r="N136" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="O136" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="137" spans="1:15" x14ac:dyDescent="0.2">
@@ -12152,7 +12171,7 @@
       <c r="B137" s="9"/>
       <c r="C137" s="9"/>
       <c r="D137" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E137" s="9"/>
       <c r="F137" s="12">
@@ -12187,7 +12206,7 @@
       <c r="B138" s="9"/>
       <c r="C138" s="9"/>
       <c r="D138" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E138" s="9"/>
       <c r="F138" s="12">
@@ -12222,7 +12241,7 @@
       <c r="B139" s="9"/>
       <c r="C139" s="9"/>
       <c r="D139" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E139" s="9"/>
       <c r="F139" s="12">
@@ -12257,32 +12276,32 @@
       <c r="B140" s="9"/>
       <c r="C140" s="9"/>
       <c r="D140" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E140" s="9"/>
       <c r="F140" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G140" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H140" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I140" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J140" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K140" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L140" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M140" s="50" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N140" s="9"/>
       <c r="O140" s="9"/>
@@ -12292,7 +12311,7 @@
       <c r="B141" s="9"/>
       <c r="C141" s="9"/>
       <c r="D141" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E141" s="9"/>
       <c r="F141" s="12">
@@ -12327,7 +12346,7 @@
       <c r="B142" s="9"/>
       <c r="C142" s="9"/>
       <c r="D142" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E142" s="9"/>
       <c r="F142" s="12">
@@ -12362,7 +12381,7 @@
       <c r="B143" s="9"/>
       <c r="C143" s="9"/>
       <c r="D143" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E143" s="9"/>
       <c r="F143" s="12">
@@ -12394,16 +12413,16 @@
     </row>
     <row r="144" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A144" s="18" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B144" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C144" s="18" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D144" s="17" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E144" s="18" t="s">
         <v>23</v>
@@ -12433,10 +12452,10 @@
         <v>1</v>
       </c>
       <c r="N144" s="18" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="O144" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="145" spans="1:15" x14ac:dyDescent="0.2">
@@ -12444,7 +12463,7 @@
       <c r="B145" s="18"/>
       <c r="C145" s="18"/>
       <c r="D145" s="17" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E145" s="18"/>
       <c r="F145" s="19">
@@ -12479,7 +12498,7 @@
       <c r="B146" s="18"/>
       <c r="C146" s="18"/>
       <c r="D146" s="17" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E146" s="18"/>
       <c r="F146" s="19">
@@ -12514,7 +12533,7 @@
       <c r="B147" s="18"/>
       <c r="C147" s="18"/>
       <c r="D147" s="17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E147" s="18"/>
       <c r="F147" s="19">
@@ -12549,7 +12568,7 @@
       <c r="B148" s="18"/>
       <c r="C148" s="18"/>
       <c r="D148" s="17" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E148" s="18"/>
       <c r="F148" s="19">
@@ -12584,7 +12603,7 @@
       <c r="B149" s="18"/>
       <c r="C149" s="18"/>
       <c r="D149" s="17" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E149" s="18"/>
       <c r="F149" s="19">
@@ -12654,7 +12673,7 @@
       <c r="B151" s="18"/>
       <c r="C151" s="18"/>
       <c r="D151" s="17" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E151" s="18"/>
       <c r="F151" s="19">
@@ -12689,7 +12708,7 @@
       <c r="B152" s="18"/>
       <c r="C152" s="18"/>
       <c r="D152" s="17" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E152" s="18"/>
       <c r="F152" s="19">
@@ -12724,7 +12743,7 @@
       <c r="B153" s="18"/>
       <c r="C153" s="18"/>
       <c r="D153" s="17" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E153" s="18"/>
       <c r="F153" s="19">
@@ -12759,7 +12778,7 @@
       <c r="B154" s="18"/>
       <c r="C154" s="18"/>
       <c r="D154" s="17" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E154" s="18"/>
       <c r="F154" s="19">
@@ -12791,16 +12810,16 @@
     </row>
     <row r="155" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="9" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B155" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C155" s="9" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D155" s="13" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>23</v>
@@ -12830,10 +12849,10 @@
         <v>1</v>
       </c>
       <c r="N155" s="9" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="O155" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="156" spans="1:15" x14ac:dyDescent="0.2">
@@ -12841,7 +12860,7 @@
       <c r="B156" s="9"/>
       <c r="C156" s="9"/>
       <c r="D156" s="13" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E156" s="9"/>
       <c r="F156" s="47">
@@ -12876,7 +12895,7 @@
       <c r="B157" s="9"/>
       <c r="C157" s="9"/>
       <c r="D157" s="13" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E157" s="9"/>
       <c r="F157" s="47">
@@ -12911,7 +12930,7 @@
       <c r="B158" s="9"/>
       <c r="C158" s="9"/>
       <c r="D158" s="13" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E158" s="9"/>
       <c r="F158" s="47">
@@ -12946,7 +12965,7 @@
       <c r="B159" s="9"/>
       <c r="C159" s="9"/>
       <c r="D159" s="13" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E159" s="9"/>
       <c r="F159" s="47">
@@ -12981,7 +13000,7 @@
       <c r="B160" s="9"/>
       <c r="C160" s="9"/>
       <c r="D160" s="13" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E160" s="9"/>
       <c r="F160" s="47">
@@ -13051,7 +13070,7 @@
       <c r="B162" s="9"/>
       <c r="C162" s="9"/>
       <c r="D162" s="13" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E162" s="9"/>
       <c r="F162" s="47">
@@ -13086,7 +13105,7 @@
       <c r="B163" s="9"/>
       <c r="C163" s="9"/>
       <c r="D163" s="13" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E163" s="9"/>
       <c r="F163" s="47">
@@ -13121,7 +13140,7 @@
       <c r="B164" s="9"/>
       <c r="C164" s="9"/>
       <c r="D164" s="13" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E164" s="9"/>
       <c r="F164" s="47">
@@ -13156,7 +13175,7 @@
       <c r="B165" s="9"/>
       <c r="C165" s="9"/>
       <c r="D165" s="13" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E165" s="9"/>
       <c r="F165" s="47">
@@ -13188,16 +13207,16 @@
     </row>
     <row r="166" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="18" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B166" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C166" s="18" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D166" s="17" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E166" s="18" t="s">
         <v>23</v>
@@ -13227,10 +13246,10 @@
         <v>1</v>
       </c>
       <c r="N166" s="18" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="O166" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="167" spans="1:15" x14ac:dyDescent="0.2">
@@ -13238,7 +13257,7 @@
       <c r="B167" s="18"/>
       <c r="C167" s="18"/>
       <c r="D167" s="17" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E167" s="18"/>
       <c r="F167" s="54">
@@ -13273,7 +13292,7 @@
       <c r="B168" s="18"/>
       <c r="C168" s="18"/>
       <c r="D168" s="17" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E168" s="18"/>
       <c r="F168" s="54">
@@ -13308,7 +13327,7 @@
       <c r="B169" s="18"/>
       <c r="C169" s="18"/>
       <c r="D169" s="17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E169" s="18"/>
       <c r="F169" s="54">
@@ -13343,7 +13362,7 @@
       <c r="B170" s="18"/>
       <c r="C170" s="18"/>
       <c r="D170" s="17" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E170" s="18"/>
       <c r="F170" s="54">
@@ -13378,7 +13397,7 @@
       <c r="B171" s="18"/>
       <c r="C171" s="18"/>
       <c r="D171" s="17" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E171" s="18"/>
       <c r="F171" s="54">
@@ -13448,7 +13467,7 @@
       <c r="B173" s="18"/>
       <c r="C173" s="18"/>
       <c r="D173" s="17" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E173" s="18"/>
       <c r="F173" s="54">
@@ -13483,7 +13502,7 @@
       <c r="B174" s="18"/>
       <c r="C174" s="18"/>
       <c r="D174" s="17" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E174" s="18"/>
       <c r="F174" s="54">
@@ -13518,7 +13537,7 @@
       <c r="B175" s="18"/>
       <c r="C175" s="18"/>
       <c r="D175" s="17" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E175" s="18"/>
       <c r="F175" s="54">
@@ -13553,7 +13572,7 @@
       <c r="B176" s="18"/>
       <c r="C176" s="18"/>
       <c r="D176" s="17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E176" s="18"/>
       <c r="F176" s="54">
@@ -13585,16 +13604,16 @@
     </row>
     <row r="177" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A177" s="46" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B177" s="46" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C177" s="46" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D177" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E177" s="46" t="s">
         <v>38</v>
@@ -13624,10 +13643,10 @@
         <v>2</v>
       </c>
       <c r="N177" s="46" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="O177" s="46" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="178" spans="1:15" x14ac:dyDescent="0.2">
@@ -13635,7 +13654,7 @@
       <c r="B178" s="46"/>
       <c r="C178" s="46"/>
       <c r="D178" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E178" s="46"/>
       <c r="F178" s="12">
@@ -13670,7 +13689,7 @@
       <c r="B179" s="46"/>
       <c r="C179" s="46"/>
       <c r="D179" s="13" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E179" s="46"/>
       <c r="F179" s="12">
@@ -13705,7 +13724,7 @@
       <c r="B180" s="46"/>
       <c r="C180" s="46"/>
       <c r="D180" s="13" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E180" s="46"/>
       <c r="F180" s="12">
@@ -13740,32 +13759,32 @@
       <c r="B181" s="46"/>
       <c r="C181" s="46"/>
       <c r="D181" s="13" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E181" s="46"/>
       <c r="F181" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G181" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H181" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I181" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J181" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K181" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L181" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M181" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N181" s="46"/>
       <c r="O181" s="46"/>
@@ -13775,7 +13794,7 @@
       <c r="B182" s="46"/>
       <c r="C182" s="46"/>
       <c r="D182" s="13" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E182" s="46"/>
       <c r="F182" s="12">
@@ -13810,7 +13829,7 @@
       <c r="B183" s="46"/>
       <c r="C183" s="46"/>
       <c r="D183" s="13" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E183" s="46"/>
       <c r="F183" s="12">
@@ -13845,7 +13864,7 @@
       <c r="B184" s="46"/>
       <c r="C184" s="46"/>
       <c r="D184" s="13" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E184" s="46"/>
       <c r="F184" s="12">
@@ -13877,16 +13896,16 @@
     </row>
     <row r="185" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A185" s="18" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B185" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C185" s="18" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D185" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E185" s="18" t="s">
         <v>38</v>
@@ -13916,10 +13935,10 @@
         <v>1</v>
       </c>
       <c r="N185" s="18" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="O185" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="186" spans="1:15" x14ac:dyDescent="0.2">
@@ -13927,7 +13946,7 @@
       <c r="B186" s="18"/>
       <c r="C186" s="18"/>
       <c r="D186" s="17" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E186" s="18"/>
       <c r="F186" s="19">
@@ -13962,7 +13981,7 @@
       <c r="B187" s="18"/>
       <c r="C187" s="18"/>
       <c r="D187" s="17" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E187" s="18"/>
       <c r="F187" s="19">
@@ -13997,7 +14016,7 @@
       <c r="B188" s="18"/>
       <c r="C188" s="18"/>
       <c r="D188" s="17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E188" s="18"/>
       <c r="F188" s="19">
@@ -14032,32 +14051,32 @@
       <c r="B189" s="18"/>
       <c r="C189" s="18"/>
       <c r="D189" s="17" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E189" s="18"/>
       <c r="F189" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G189" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H189" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I189" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J189" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K189" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L189" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M189" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N189" s="18"/>
       <c r="O189" s="18"/>
@@ -14067,7 +14086,7 @@
       <c r="B190" s="18"/>
       <c r="C190" s="18"/>
       <c r="D190" s="17" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E190" s="18"/>
       <c r="F190" s="19">
@@ -14102,7 +14121,7 @@
       <c r="B191" s="18"/>
       <c r="C191" s="18"/>
       <c r="D191" s="17" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E191" s="18"/>
       <c r="F191" s="19">
@@ -14137,7 +14156,7 @@
       <c r="B192" s="18"/>
       <c r="C192" s="18"/>
       <c r="D192" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E192" s="18"/>
       <c r="F192" s="19">
@@ -14169,16 +14188,16 @@
     </row>
     <row r="193" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B193" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C193" s="9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D193" s="13" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E193" s="9" t="s">
         <v>23</v>
@@ -14208,10 +14227,10 @@
         <v>2</v>
       </c>
       <c r="N193" s="9" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="O193" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="194" spans="1:15" x14ac:dyDescent="0.2">
@@ -14219,7 +14238,7 @@
       <c r="B194" s="9"/>
       <c r="C194" s="9"/>
       <c r="D194" s="13" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E194" s="9"/>
       <c r="F194" s="10">
@@ -14254,7 +14273,7 @@
       <c r="B195" s="9"/>
       <c r="C195" s="9"/>
       <c r="D195" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E195" s="9"/>
       <c r="F195" s="10">
@@ -14289,7 +14308,7 @@
       <c r="B196" s="9"/>
       <c r="C196" s="9"/>
       <c r="D196" s="13" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E196" s="9"/>
       <c r="F196" s="10">
@@ -14324,7 +14343,7 @@
       <c r="B197" s="9"/>
       <c r="C197" s="9"/>
       <c r="D197" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E197" s="9"/>
       <c r="F197" s="12">
@@ -14359,7 +14378,7 @@
       <c r="B198" s="9"/>
       <c r="C198" s="9"/>
       <c r="D198" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E198" s="9"/>
       <c r="F198" s="12">
@@ -14394,7 +14413,7 @@
       <c r="B199" s="9"/>
       <c r="C199" s="9"/>
       <c r="D199" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E199" s="9"/>
       <c r="F199" s="12">
@@ -14429,7 +14448,7 @@
       <c r="B200" s="9"/>
       <c r="C200" s="9"/>
       <c r="D200" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E200" s="9"/>
       <c r="F200" s="12">
@@ -14464,32 +14483,32 @@
       <c r="B201" s="9"/>
       <c r="C201" s="9"/>
       <c r="D201" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E201" s="9"/>
       <c r="F201" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G201" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H201" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J201" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K201" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L201" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M201" s="53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N201" s="9"/>
       <c r="O201" s="9"/>
@@ -14499,7 +14518,7 @@
       <c r="B202" s="9"/>
       <c r="C202" s="9"/>
       <c r="D202" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E202" s="9"/>
       <c r="F202" s="12">
@@ -14534,7 +14553,7 @@
       <c r="B203" s="9"/>
       <c r="C203" s="9"/>
       <c r="D203" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E203" s="9"/>
       <c r="F203" s="12">
@@ -14569,7 +14588,7 @@
       <c r="B204" s="9"/>
       <c r="C204" s="9"/>
       <c r="D204" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E204" s="9"/>
       <c r="F204" s="12">
@@ -14601,16 +14620,16 @@
     </row>
     <row r="205" spans="1:15" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="18" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B205" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C205" s="18" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D205" s="17" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E205" s="18" t="s">
         <v>23</v>
@@ -14640,10 +14659,10 @@
         <v>1</v>
       </c>
       <c r="N205" s="18" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="O205" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="206" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -14651,7 +14670,7 @@
       <c r="B206" s="18"/>
       <c r="C206" s="18"/>
       <c r="D206" s="17" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E206" s="18"/>
       <c r="F206" s="19">
@@ -14686,7 +14705,7 @@
       <c r="B207" s="18"/>
       <c r="C207" s="18"/>
       <c r="D207" s="17" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E207" s="18"/>
       <c r="F207" s="19">
@@ -14721,7 +14740,7 @@
       <c r="B208" s="18"/>
       <c r="C208" s="18"/>
       <c r="D208" s="17" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E208" s="18"/>
       <c r="F208" s="19">
@@ -14756,7 +14775,7 @@
       <c r="B209" s="18"/>
       <c r="C209" s="18"/>
       <c r="D209" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E209" s="18"/>
       <c r="F209" s="19">
@@ -14791,7 +14810,7 @@
       <c r="B210" s="18"/>
       <c r="C210" s="18"/>
       <c r="D210" s="17" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E210" s="18"/>
       <c r="F210" s="19">
@@ -14826,7 +14845,7 @@
       <c r="B211" s="18"/>
       <c r="C211" s="18"/>
       <c r="D211" s="17" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E211" s="18"/>
       <c r="F211" s="19">
@@ -14861,7 +14880,7 @@
       <c r="B212" s="18"/>
       <c r="C212" s="18"/>
       <c r="D212" s="17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E212" s="18"/>
       <c r="F212" s="19">
@@ -14896,32 +14915,32 @@
       <c r="B213" s="18"/>
       <c r="C213" s="18"/>
       <c r="D213" s="17" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E213" s="18"/>
       <c r="F213" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G213" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H213" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I213" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J213" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="K213" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="L213" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M213" s="49" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="N213" s="18"/>
       <c r="O213" s="18"/>
@@ -14931,7 +14950,7 @@
       <c r="B214" s="18"/>
       <c r="C214" s="18"/>
       <c r="D214" s="17" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E214" s="18"/>
       <c r="F214" s="19">
@@ -14966,7 +14985,7 @@
       <c r="B215" s="18"/>
       <c r="C215" s="18"/>
       <c r="D215" s="17" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E215" s="18"/>
       <c r="F215" s="19">
@@ -15001,7 +15020,7 @@
       <c r="B216" s="18"/>
       <c r="C216" s="18"/>
       <c r="D216" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E216" s="18"/>
       <c r="F216" s="19">
@@ -15204,24 +15223,24 @@
   <sheetData>
     <row r="2" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D2" s="34" t="s">
+        <v>265</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="G2" s="34" t="s">
         <v>268</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>269</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>270</v>
-      </c>
-      <c r="G2" s="34" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="3" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C3" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D3">
         <v>25</v>
@@ -15238,7 +15257,7 @@
     </row>
     <row r="4" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D4">
         <v>11</v>
@@ -15249,7 +15268,7 @@
     </row>
     <row r="5" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -15260,7 +15279,7 @@
     </row>
     <row r="6" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D6">
         <v>11</v>
@@ -15271,7 +15290,7 @@
     </row>
     <row r="7" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D7">
         <v>17</v>
@@ -15282,7 +15301,13 @@
     </row>
     <row r="8" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
-        <v>278</v>
+        <v>275</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>